<commit_message>
Upload schedule from GitHub Pages: Schedule TS.xlsx
</commit_message>
<xml_diff>
--- a/uploads/Schedule.xlsx
+++ b/uploads/Schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iafid-my.sharepoint.com/personal/cahya_rimbawan_iaf_co_id/Documents/DOC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{74F4ADBB-4B30-4BD8-A417-8FF76D47880D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{83404A6E-490E-448B-939B-195A5B27E7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="3" activeTab="3" xr2:uid="{CE6A7F6E-43F7-460E-93E3-39822A35E0CD}"/>
   </bookViews>
@@ -348,7 +348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -432,13 +432,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -782,51 +776,51 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="21">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
     </row>
     <row r="4" spans="2:10">
-      <c r="B4" s="47" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="47" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="48" t="s">
+      <c r="B4" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="46"/>
     </row>
     <row r="5" spans="2:10">
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
       <c r="D5" s="5"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
@@ -842,8 +836,8 @@
       </c>
     </row>
     <row r="6" spans="2:10">
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
       <c r="D6" s="5"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -904,10 +898,10 @@
       <c r="J9" s="2"/>
     </row>
     <row r="10" spans="2:10">
-      <c r="B10" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C10" s="42" t="s">
+      <c r="B10" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="5" t="s">
@@ -933,8 +927,8 @@
       </c>
     </row>
     <row r="11" spans="2:10">
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="41"/>
       <c r="D11" s="5">
         <v>13</v>
       </c>
@@ -1003,10 +997,10 @@
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" s="42" t="s">
+      <c r="B15" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -1032,8 +1026,8 @@
       </c>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="43"/>
-      <c r="C16" s="43"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="41"/>
       <c r="D16" s="5">
         <v>20</v>
       </c>
@@ -1101,10 +1095,10 @@
       <c r="J19" s="19"/>
     </row>
     <row r="20" spans="2:10">
-      <c r="B20" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C20" s="42" t="s">
+      <c r="B20" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D20" s="5" t="s">
@@ -1124,8 +1118,8 @@
       <c r="J20" s="18"/>
     </row>
     <row r="21" spans="2:10">
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
+      <c r="B21" s="41"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="5">
         <v>27</v>
       </c>
@@ -1253,51 +1247,51 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="21">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
     </row>
     <row r="4" spans="2:10">
-      <c r="B4" s="47" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="47" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="48" t="s">
+      <c r="B4" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="46"/>
     </row>
     <row r="5" spans="2:10">
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
       <c r="D5" s="5"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
@@ -1313,8 +1307,8 @@
       </c>
     </row>
     <row r="6" spans="2:10">
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
       <c r="D6" s="5"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -1375,10 +1369,10 @@
       <c r="J9" s="2"/>
     </row>
     <row r="10" spans="2:10">
-      <c r="B10" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C10" s="42" t="s">
+      <c r="B10" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="5" t="s">
@@ -1404,8 +1398,8 @@
       </c>
     </row>
     <row r="11" spans="2:10">
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="41"/>
       <c r="D11" s="5">
         <v>4</v>
       </c>
@@ -1474,10 +1468,10 @@
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" s="42" t="s">
+      <c r="B15" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -1503,8 +1497,8 @@
       </c>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="43"/>
-      <c r="C16" s="43"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="41"/>
       <c r="D16" s="5">
         <v>11</v>
       </c>
@@ -1572,10 +1566,10 @@
       <c r="J19" s="27"/>
     </row>
     <row r="20" spans="2:21">
-      <c r="B20" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C20" s="42" t="s">
+      <c r="B20" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D20" s="5" t="s">
@@ -1601,8 +1595,8 @@
       </c>
     </row>
     <row r="21" spans="2:21">
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
+      <c r="B21" s="41"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="5">
         <v>18</v>
       </c>
@@ -1671,10 +1665,10 @@
       <c r="J24" s="2"/>
     </row>
     <row r="25" spans="2:21">
-      <c r="B25" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C25" s="42" t="s">
+      <c r="B25" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D25" s="5" t="s">
@@ -1700,8 +1694,8 @@
       </c>
     </row>
     <row r="26" spans="2:21">
-      <c r="B26" s="43"/>
-      <c r="C26" s="43"/>
+      <c r="B26" s="41"/>
+      <c r="C26" s="41"/>
       <c r="D26" s="5">
         <v>25</v>
       </c>
@@ -1877,51 +1871,51 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="21">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
     </row>
     <row r="4" spans="2:10">
-      <c r="B4" s="47" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="47" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="48" t="s">
+      <c r="B4" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="46"/>
     </row>
     <row r="5" spans="2:10">
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
       <c r="D5" s="6" t="s">
         <v>11</v>
       </c>
@@ -1945,8 +1939,8 @@
       </c>
     </row>
     <row r="6" spans="2:10">
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
       <c r="D6" s="6">
         <v>1</v>
       </c>
@@ -2015,10 +2009,10 @@
       <c r="J9" s="8"/>
     </row>
     <row r="10" spans="2:10">
-      <c r="B10" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C10" s="42" t="s">
+      <c r="B10" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="5" t="s">
@@ -2044,8 +2038,8 @@
       </c>
     </row>
     <row r="11" spans="2:10">
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="41"/>
       <c r="D11" s="5">
         <v>8</v>
       </c>
@@ -2114,10 +2108,10 @@
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" s="42" t="s">
+      <c r="B15" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -2143,8 +2137,8 @@
       </c>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="43"/>
-      <c r="C16" s="43"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="41"/>
       <c r="D16" s="5">
         <v>15</v>
       </c>
@@ -2212,10 +2206,10 @@
       <c r="J19" s="34"/>
     </row>
     <row r="20" spans="2:21">
-      <c r="B20" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C20" s="42" t="s">
+      <c r="B20" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D20" s="5" t="s">
@@ -2241,8 +2235,8 @@
       </c>
     </row>
     <row r="21" spans="2:21">
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
+      <c r="B21" s="41"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="5">
         <v>22</v>
       </c>
@@ -2311,10 +2305,10 @@
       <c r="J24" s="8"/>
     </row>
     <row r="25" spans="2:21">
-      <c r="B25" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C25" s="42" t="s">
+      <c r="B25" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D25" s="5" t="s">
@@ -2330,8 +2324,8 @@
       <c r="J25" s="35"/>
     </row>
     <row r="26" spans="2:21">
-      <c r="B26" s="43"/>
-      <c r="C26" s="43"/>
+      <c r="B26" s="41"/>
+      <c r="C26" s="41"/>
       <c r="D26" s="5">
         <v>29</v>
       </c>
@@ -2497,51 +2491,51 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="21">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
     </row>
     <row r="3" spans="2:10">
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
     </row>
     <row r="4" spans="2:10">
-      <c r="B4" s="47" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="47" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="48" t="s">
+      <c r="B4" s="45" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="46"/>
     </row>
     <row r="5" spans="2:10">
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
       <c r="D5" s="6"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5" t="s">
@@ -2561,8 +2555,8 @@
       </c>
     </row>
     <row r="6" spans="2:10">
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
       <c r="D6" s="6"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5">
@@ -2620,17 +2614,17 @@
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="40"/>
+      <c r="F9" s="39"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9"/>
       <c r="I9" s="8"/>
       <c r="J9" s="2"/>
     </row>
     <row r="10" spans="2:10">
-      <c r="B10" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C10" s="42" t="s">
+      <c r="B10" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="5" t="s">
@@ -2656,8 +2650,8 @@
       </c>
     </row>
     <row r="11" spans="2:10">
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="41"/>
       <c r="D11" s="5">
         <v>6</v>
       </c>
@@ -2689,7 +2683,7 @@
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
+      <c r="F12" s="17"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="8"/>
@@ -2717,7 +2711,7 @@
       <c r="C14" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="41"/>
+      <c r="D14" s="33"/>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
@@ -2726,10 +2720,10 @@
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" s="42" t="s">
+      <c r="B15" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -2755,8 +2749,8 @@
       </c>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="43"/>
-      <c r="C16" s="43"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="41"/>
       <c r="D16" s="5">
         <v>13</v>
       </c>
@@ -2790,7 +2784,7 @@
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
+      <c r="H17" s="17"/>
       <c r="J17" s="2"/>
     </row>
     <row r="18" spans="2:21">
@@ -2802,11 +2796,11 @@
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="F18" s="17"/>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="39"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="21"/>
     </row>
     <row r="19" spans="2:21">
       <c r="B19" s="2">
@@ -2820,14 +2814,14 @@
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="34"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="27"/>
     </row>
     <row r="20" spans="2:21">
-      <c r="B20" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C20" s="42" t="s">
+      <c r="B20" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D20" s="5" t="s">
@@ -2853,8 +2847,8 @@
       </c>
     </row>
     <row r="21" spans="2:21">
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
+      <c r="B21" s="41"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="5">
         <v>20</v>
       </c>
@@ -2904,7 +2898,7 @@
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="8"/>
+      <c r="I23" s="2"/>
       <c r="J23" s="2"/>
     </row>
     <row r="24" spans="2:21">
@@ -2919,14 +2913,14 @@
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
       <c r="H24" s="9"/>
-      <c r="I24" s="2"/>
+      <c r="I24" s="8"/>
       <c r="J24" s="2"/>
     </row>
     <row r="25" spans="2:21">
-      <c r="B25" s="42" t="s">
-        <v>2</v>
-      </c>
-      <c r="C25" s="42" t="s">
+      <c r="B25" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25" s="40" t="s">
         <v>3</v>
       </c>
       <c r="D25" s="5" t="s">
@@ -2948,8 +2942,8 @@
       <c r="J25" s="5"/>
     </row>
     <row r="26" spans="2:21">
-      <c r="B26" s="43"/>
-      <c r="C26" s="43"/>
+      <c r="B26" s="41"/>
+      <c r="C26" s="41"/>
       <c r="D26" s="5">
         <v>27</v>
       </c>
@@ -3112,17 +3106,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ac6e70c6-6e36-4426-b8b7-4d7d3edbc74e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="27ddc5ee-c3d9-45fc-a76d-ba15e8ec9144" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010062FAB611ECDA514281B08A367BBFEC58" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5569e5f6b0f0d8e749239d749d7049d2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ac6e70c6-6e36-4426-b8b7-4d7d3edbc74e" xmlns:ns3="27ddc5ee-c3d9-45fc-a76d-ba15e8ec9144" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ba38082228e24ce3e127784df4a0bb2a" ns2:_="" ns3:_="">
     <xsd:import namespace="ac6e70c6-6e36-4426-b8b7-4d7d3edbc74e"/>
@@ -3357,7 +3340,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3366,14 +3349,25 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ac6e70c6-6e36-4426-b8b7-4d7d3edbc74e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="27ddc5ee-c3d9-45fc-a76d-ba15e8ec9144" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78395C7D-0FE3-4B64-BBC9-94773B0377B5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F080A64-874E-499C-996B-84204DB4DD2B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F080A64-874E-499C-996B-84204DB4DD2B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4920AA2F-2305-4E6E-89EB-700F99738508}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4920AA2F-2305-4E6E-89EB-700F99738508}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78395C7D-0FE3-4B64-BBC9-94773B0377B5}"/>
 </file>
</xml_diff>